<commit_message>
feat: add critical GI management pages and sample CSV template for inspection data
</commit_message>
<xml_diff>
--- a/hifi-power-inspect/Master/template_critical_gi.xlsx
+++ b/hifi-power-inspect/Master/template_critical_gi.xlsx
@@ -456,7 +456,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
@@ -519,7 +519,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>GI 150kV UJUNG BERUNG</t>
+          <t>GI 150KV UJUNGBERUNG</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>GI 150kV CIGERELENG</t>
+          <t>GI 150KV CIGERELENG</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>GI 150kV SUNJAYARAGI</t>
+          <t>GI 150KV SUNYARAGI</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>GI 150kV KOSAMBI</t>
+          <t>GI 150KV KOSAMBI</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>GI 150kV TELUK JAMBE</t>
+          <t>GI 150KV TELUKJAMBE</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">

</xml_diff>